<commit_message>
Added Sea Breeze,Gold_view,Ft Lauderdale test data
</commit_message>
<xml_diff>
--- a/output/Coastal/Cash_Reconciliation_Report.xlsx
+++ b/output/Coastal/Cash_Reconciliation_Report.xlsx
@@ -423,10 +423,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>COASTAL CENTER OPERATIONS LLC MONOGRAM CHECKING 1503764063:</v>
+        <v>RFMS Account # ****6932:</v>
       </c>
       <c r="B3" t="str">
-        <v>$45,306.12</v>
+        <v>$26,600.77</v>
       </c>
       <c r="C3" t="str">
         <v/>
@@ -434,10 +434,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>COASTAL CENTER OPERATIONS NON-GOVERNMENT RECEIVABLE XXXXXXXX3858:</v>
+        <v>Coastal Center Operations LLC MONOGRAM CHECKING 1503764063:</v>
       </c>
       <c r="B4" t="str">
-        <v>$917,172.99</v>
+        <v>$45,306.12</v>
       </c>
       <c r="C4" t="str">
         <v/>
@@ -456,10 +456,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>RFMS Account # ****6932:</v>
+        <v>NON-GOVERNMENT RECEIVABLE XXXXXXXX3858:</v>
       </c>
       <c r="B6" t="str">
-        <v>$26,600.77</v>
+        <v>$917,172.99</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -528,7 +528,7 @@
         <v>Sunshine Really$0.00</v>
       </c>
       <c r="C12" t="str">
-        <v>$-359.69</v>
+        <v>-$359.69</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Modified login and reload according to the chnaged ui
</commit_message>
<xml_diff>
--- a/output/Coastal/Cash_Reconciliation_Report.xlsx
+++ b/output/Coastal/Cash_Reconciliation_Report.xlsx
@@ -434,7 +434,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Coastal Center Operations LLC MONOGRAM CHECKING 1503764063:</v>
+        <v>MONOGRAM CHECKING 1503764063:</v>
       </c>
       <c r="B4" t="str">
         <v>$45,306.12</v>
@@ -456,7 +456,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Coastal Center Operations LLC NON-GOVERNMENT RECEIVABLE XXXXXXXX3858:</v>
+        <v>NON-GOVERNMENT RECEIVABLE XXXXXXXX3858:</v>
       </c>
       <c r="B6" t="str">
         <v>$917,172.99</v>

</xml_diff>